<commit_message>
preparar plan optimizacion rendimiento
</commit_message>
<xml_diff>
--- a/oportunidad-generar-core-main/data/output/CORE_AT_20251160543.xlsx
+++ b/oportunidad-generar-core-main/data/output/CORE_AT_20251160543.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aortega\.nuget\packages\oportunidad-generar-core-main\1.0.37-rpa-validacion\content\data\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aortega\Documents\UiPath\oportunidad-generar-core-v3\oportunidad-generar-core-main\data\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C74B67A3-6A6A-49CB-A254-348C7EA28637}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF9FD339-CB6D-4DC4-A0BA-BC566EC3CFE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="669" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1123,7 +1123,7 @@
     <t>Sopore especializado</t>
   </si>
   <si>
-    <t>RPA_VALIDACION: Generado por RPA: 2026-05-12 00:26:08 | PPO=20251160543_PPO_CEducación_AMS_SI_Lote 2_v01.xlsm | NumeroSF=20251160543 | Tipo=AT | Campos PPO=8 | Trazabilidad: PPO=baseline; SAP/SF=datos de prueba hardcodeados en Main.xaml; reglas=recursos/gastos/compras prorrateados por anualidad, riesgos/garantia al ultimo mes, facturacion y realizado vacios; pendiente JP=revisar intercompany, externos y planificacion mensual. | AT: tarifas de venta reescaladas proporcionalmente para cuadrar venta facturable con importe total de venta del proyecto: 465.000,00 EUR. Se conservan horas, costes y perfiles; solo se ajusta tarifa de venta. Revisión requerida si negocio exige tarifa literal por linea PPO.</t>
+    <t>RPA_VALIDACION: Generado por RPA: 2026-05-12 01:04:41 | PPO=20251160543_PPO_CEducación_AMS_SI_Lote 2_v01.xlsm | NumeroSF=20251160543 | Tipo=AT | Campos PPO=8 | Trazabilidad: PPO=baseline; SAP/SF=datos de prueba hardcodeados en Main.xaml; reglas=recursos/gastos/compras prorrateados por anualidad, riesgos/garantia al ultimo mes, facturacion y realizado vacios; pendiente JP=revisar intercompany, externos y planificacion mensual. | AT: tarifas de venta reescaladas proporcionalmente para cuadrar venta facturable con importe total de venta del proyecto: 465.000,00 EUR. Se conservan horas, costes y perfiles; solo se ajusta tarifa de venta. Revisión requerida si negocio exige tarifa literal por linea PPO.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
plan rendimiento - e1
</commit_message>
<xml_diff>
--- a/oportunidad-generar-core-main/data/output/CORE_AT_20251160543.xlsx
+++ b/oportunidad-generar-core-main/data/output/CORE_AT_20251160543.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aortega\Documents\UiPath\oportunidad-generar-core-v3\oportunidad-generar-core-main\data\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aortega\.nuget\packages\oportunidad-generar-core-main\1.0.38-ep1\content\data\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF9FD339-CB6D-4DC4-A0BA-BC566EC3CFE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{359449EC-3436-4D92-9A48-D931A550B9E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="669" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1123,7 +1123,7 @@
     <t>Sopore especializado</t>
   </si>
   <si>
-    <t>RPA_VALIDACION: Generado por RPA: 2026-05-12 01:04:41 | PPO=20251160543_PPO_CEducación_AMS_SI_Lote 2_v01.xlsm | NumeroSF=20251160543 | Tipo=AT | Campos PPO=8 | Trazabilidad: PPO=baseline; SAP/SF=datos de prueba hardcodeados en Main.xaml; reglas=recursos/gastos/compras prorrateados por anualidad, riesgos/garantia al ultimo mes, facturacion y realizado vacios; pendiente JP=revisar intercompany, externos y planificacion mensual. | AT: tarifas de venta reescaladas proporcionalmente para cuadrar venta facturable con importe total de venta del proyecto: 465.000,00 EUR. Se conservan horas, costes y perfiles; solo se ajusta tarifa de venta. Revisión requerida si negocio exige tarifa literal por linea PPO.</t>
+    <t>RPA_VALIDACION: Generado por RPA: 2026-05-12 02:12:49 | PPO=20251160543_PPO_CEducación_AMS_SI_Lote 2_v01.xlsm | NumeroSF=20251160543 | Tipo=AT | Campos PPO=8 | Trazabilidad: PPO=baseline; SAP/SF=datos de prueba hardcodeados en Main.xaml; reglas=recursos/gastos/compras prorrateados por anualidad, riesgos/garantia al ultimo mes, facturacion y realizado vacios; pendiente JP=revisar intercompany, externos y planificacion mensual. | AT: tarifas de venta reescaladas proporcionalmente para cuadrar venta facturable con importe total de venta del proyecto: 465.000,00 EUR. Se conservan horas, costes y perfiles; solo se ajusta tarifa de venta. Revisión requerida si negocio exige tarifa literal por linea PPO.</t>
   </si>
 </sst>
 </file>
@@ -3072,6 +3072,13 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -3081,16 +3088,9 @@
     <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="164" fontId="11" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -9016,7 +9016,7 @@
       </c>
       <c r="D4" s="315"/>
       <c r="E4" s="22"/>
-      <c r="F4" s="332" t="s">
+      <c r="F4" s="328" t="s">
         <v>238</v>
       </c>
       <c r="G4" s="333"/>
@@ -9029,26 +9029,26 @@
       <c r="J4" s="228" t="s">
         <v>241</v>
       </c>
-      <c r="K4" s="332" t="s">
+      <c r="K4" s="328" t="s">
         <v>242</v>
       </c>
-      <c r="L4" s="332"/>
-      <c r="M4" s="332"/>
-      <c r="N4" s="332"/>
+      <c r="L4" s="328"/>
+      <c r="M4" s="328"/>
+      <c r="N4" s="328"/>
     </row>
     <row r="5" spans="2:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="77" t="s">
         <v>243</v>
       </c>
-      <c r="C5" s="330" t="s">
+      <c r="C5" s="327" t="s">
         <v>244</v>
       </c>
-      <c r="D5" s="330"/>
+      <c r="D5" s="327"/>
       <c r="E5" s="22"/>
-      <c r="F5" s="330" t="s">
+      <c r="F5" s="327" t="s">
         <v>245</v>
       </c>
-      <c r="G5" s="330"/>
+      <c r="G5" s="327"/>
       <c r="H5" s="230">
         <v>0.5</v>
       </c>
@@ -9058,24 +9058,24 @@
       <c r="J5" s="289" t="s">
         <v>244</v>
       </c>
-      <c r="K5" s="330"/>
-      <c r="L5" s="330"/>
-      <c r="M5" s="330"/>
-      <c r="N5" s="330"/>
+      <c r="K5" s="327"/>
+      <c r="L5" s="327"/>
+      <c r="M5" s="327"/>
+      <c r="N5" s="327"/>
     </row>
     <row r="6" spans="2:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="77" t="s">
         <v>246</v>
       </c>
-      <c r="C6" s="330" t="s">
+      <c r="C6" s="327" t="s">
         <v>247</v>
       </c>
-      <c r="D6" s="330"/>
+      <c r="D6" s="327"/>
       <c r="E6" s="22"/>
-      <c r="F6" s="330" t="s">
+      <c r="F6" s="327" t="s">
         <v>248</v>
       </c>
-      <c r="G6" s="330"/>
+      <c r="G6" s="327"/>
       <c r="H6" s="230">
         <v>0.1</v>
       </c>
@@ -9083,26 +9083,26 @@
         <v>1000</v>
       </c>
       <c r="J6" s="289"/>
-      <c r="K6" s="330"/>
-      <c r="L6" s="330"/>
-      <c r="M6" s="330"/>
-      <c r="N6" s="330"/>
+      <c r="K6" s="327"/>
+      <c r="L6" s="327"/>
+      <c r="M6" s="327"/>
+      <c r="N6" s="327"/>
     </row>
     <row r="7" spans="2:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="77" t="s">
         <v>249</v>
       </c>
-      <c r="C7" s="331">
+      <c r="C7" s="332">
         <v>10000</v>
       </c>
-      <c r="D7" s="331"/>
+      <c r="D7" s="332"/>
       <c r="E7" s="229" t="s">
         <v>250</v>
       </c>
-      <c r="F7" s="330" t="s">
+      <c r="F7" s="327" t="s">
         <v>251</v>
       </c>
-      <c r="G7" s="330"/>
+      <c r="G7" s="327"/>
       <c r="H7" s="230">
         <v>0.2</v>
       </c>
@@ -9110,18 +9110,18 @@
         <v>2000</v>
       </c>
       <c r="J7" s="289"/>
-      <c r="K7" s="330"/>
-      <c r="L7" s="330"/>
-      <c r="M7" s="330"/>
-      <c r="N7" s="330"/>
+      <c r="K7" s="327"/>
+      <c r="L7" s="327"/>
+      <c r="M7" s="327"/>
+      <c r="N7" s="327"/>
     </row>
     <row r="8" spans="2:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D8" s="22"/>
       <c r="E8" s="22"/>
-      <c r="F8" s="330" t="s">
+      <c r="F8" s="327" t="s">
         <v>252</v>
       </c>
-      <c r="G8" s="330"/>
+      <c r="G8" s="327"/>
       <c r="H8" s="230">
         <v>0.1</v>
       </c>
@@ -9129,18 +9129,18 @@
         <v>1000</v>
       </c>
       <c r="J8" s="289"/>
-      <c r="K8" s="330"/>
-      <c r="L8" s="330"/>
-      <c r="M8" s="330"/>
-      <c r="N8" s="330"/>
+      <c r="K8" s="327"/>
+      <c r="L8" s="327"/>
+      <c r="M8" s="327"/>
+      <c r="N8" s="327"/>
     </row>
     <row r="9" spans="2:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D9" s="22"/>
       <c r="E9" s="56"/>
-      <c r="F9" s="330" t="s">
+      <c r="F9" s="327" t="s">
         <v>253</v>
       </c>
-      <c r="G9" s="330"/>
+      <c r="G9" s="327"/>
       <c r="H9" s="230">
         <v>0.1</v>
       </c>
@@ -9148,10 +9148,10 @@
         <v>1000</v>
       </c>
       <c r="J9" s="289"/>
-      <c r="K9" s="330"/>
-      <c r="L9" s="330"/>
-      <c r="M9" s="330"/>
-      <c r="N9" s="330"/>
+      <c r="K9" s="327"/>
+      <c r="L9" s="327"/>
+      <c r="M9" s="327"/>
+      <c r="N9" s="327"/>
       <c r="O9" s="24"/>
       <c r="P9" s="24"/>
     </row>
@@ -10237,12 +10237,12 @@
       <c r="W45" s="21"/>
     </row>
     <row r="46" spans="2:23" s="89" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="327" t="s">
+      <c r="B46" s="329" t="s">
         <v>233</v>
       </c>
-      <c r="C46" s="327"/>
-      <c r="D46" s="327"/>
-      <c r="E46" s="327"/>
+      <c r="C46" s="329"/>
+      <c r="D46" s="329"/>
+      <c r="E46" s="329"/>
       <c r="F46" s="219">
         <f>SUM(F13:F45)</f>
         <v>3000</v>
@@ -10406,16 +10406,16 @@
       <c r="R55" s="24"/>
     </row>
     <row r="56" spans="2:22" ht="285.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="328" t="s">
+      <c r="B56" s="330" t="s">
         <v>85</v>
       </c>
-      <c r="C56" s="329"/>
-      <c r="D56" s="329"/>
-      <c r="E56" s="329"/>
-      <c r="F56" s="329"/>
-      <c r="G56" s="329"/>
-      <c r="H56" s="329"/>
-      <c r="I56" s="329"/>
+      <c r="C56" s="331"/>
+      <c r="D56" s="331"/>
+      <c r="E56" s="331"/>
+      <c r="F56" s="331"/>
+      <c r="G56" s="331"/>
+      <c r="H56" s="331"/>
+      <c r="I56" s="331"/>
       <c r="J56" s="173"/>
       <c r="K56" s="173"/>
       <c r="L56" s="173"/>
@@ -10429,16 +10429,6 @@
   </sheetData>
   <autoFilter ref="B12:E12" xr:uid="{F0215733-3491-41E7-AEDA-44D9E214180D}"/>
   <mergeCells count="19">
-    <mergeCell ref="K9:N9"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="K4:N4"/>
-    <mergeCell ref="K5:N5"/>
-    <mergeCell ref="K6:N6"/>
-    <mergeCell ref="K7:N7"/>
-    <mergeCell ref="K8:N8"/>
     <mergeCell ref="B46:E46"/>
     <mergeCell ref="B56:I56"/>
     <mergeCell ref="C4:D4"/>
@@ -10448,6 +10438,16 @@
     <mergeCell ref="F5:G5"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="C10:D10"/>
+    <mergeCell ref="K4:N4"/>
+    <mergeCell ref="K5:N5"/>
+    <mergeCell ref="K6:N6"/>
+    <mergeCell ref="K7:N7"/>
+    <mergeCell ref="K8:N8"/>
+    <mergeCell ref="K9:N9"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="C10">
@@ -43020,21 +43020,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005104B4C06FD53E4DA82687A05841D03F" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f48deddc6bffdc45fb3ed0ec71e33c6c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7dc5af80-ab8f-4cff-b7cb-3463b3238b39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a8808579f8fa9f9643be1385777e037d" ns2:_="">
     <xsd:import namespace="7dc5af80-ab8f-4cff-b7cb-3463b3238b39"/>
@@ -43208,24 +43193,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4453D5CC-2F3C-48AA-8382-954EB2322467}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{794A36B1-E557-480A-80A5-281FC452AC8A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F36A1B76-9E34-462B-9C68-1BC8027D2211}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -43243,6 +43226,23 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{794A36B1-E557-480A-80A5-281FC452AC8A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4453D5CC-2F3C-48AA-8382-954EB2322467}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{040b5de6-6e2e-46f2-bca1-507eb809bbf7}" enabled="1" method="Privileged" siteId="{56d7daaa-b378-45b3-aa11-af9402b401b9}" contentBits="0" removed="0"/>

</xml_diff>

<commit_message>
plan rendimiento - e2
</commit_message>
<xml_diff>
--- a/oportunidad-generar-core-main/data/output/CORE_AT_20251160543.xlsx
+++ b/oportunidad-generar-core-main/data/output/CORE_AT_20251160543.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aortega\.nuget\packages\oportunidad-generar-core-main\1.0.38-ep1\content\data\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aortega\.nuget\packages\oportunidad-generar-core-main\1.0.39-ep2\content\data\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{359449EC-3436-4D92-9A48-D931A550B9E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74AE00AE-FEE9-413F-A984-A9CE5A16E86D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="669" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1123,7 +1123,7 @@
     <t>Sopore especializado</t>
   </si>
   <si>
-    <t>RPA_VALIDACION: Generado por RPA: 2026-05-12 02:12:49 | PPO=20251160543_PPO_CEducación_AMS_SI_Lote 2_v01.xlsm | NumeroSF=20251160543 | Tipo=AT | Campos PPO=8 | Trazabilidad: PPO=baseline; SAP/SF=datos de prueba hardcodeados en Main.xaml; reglas=recursos/gastos/compras prorrateados por anualidad, riesgos/garantia al ultimo mes, facturacion y realizado vacios; pendiente JP=revisar intercompany, externos y planificacion mensual. | AT: tarifas de venta reescaladas proporcionalmente para cuadrar venta facturable con importe total de venta del proyecto: 465.000,00 EUR. Se conservan horas, costes y perfiles; solo se ajusta tarifa de venta. Revisión requerida si negocio exige tarifa literal por linea PPO.</t>
+    <t>RPA_VALIDACION: Generado por RPA: 2026-05-12 02:29:18 | PPO=20251160543_PPO_CEducación_AMS_SI_Lote 2_v01.xlsm | NumeroSF=20251160543 | Tipo=AT | Campos PPO=8 | Trazabilidad: PPO=baseline; SAP/SF=datos de prueba hardcodeados en Main.xaml; reglas=recursos/gastos/compras prorrateados por anualidad, riesgos/garantia al ultimo mes, facturacion y realizado vacios; pendiente JP=revisar intercompany, externos y planificacion mensual. | AT: tarifas de venta reescaladas proporcionalmente para cuadrar venta facturable con importe total de venta del proyecto: 465.000,00 EUR. Se conservan horas, costes y perfiles; solo se ajusta tarifa de venta. Revisión requerida si negocio exige tarifa literal por linea PPO.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
plan rendimiento - e3
</commit_message>
<xml_diff>
--- a/oportunidad-generar-core-main/data/output/CORE_AT_20251160543.xlsx
+++ b/oportunidad-generar-core-main/data/output/CORE_AT_20251160543.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aortega\.nuget\packages\oportunidad-generar-core-main\1.0.39-ep2\content\data\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aortega\.nuget\packages\oportunidad-generar-core-main\1.0.40-ep3\content\data\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74AE00AE-FEE9-413F-A984-A9CE5A16E86D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BF60F04-87A1-434F-BDDA-F5CAD84520E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="669" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1123,7 +1123,7 @@
     <t>Sopore especializado</t>
   </si>
   <si>
-    <t>RPA_VALIDACION: Generado por RPA: 2026-05-12 02:29:18 | PPO=20251160543_PPO_CEducación_AMS_SI_Lote 2_v01.xlsm | NumeroSF=20251160543 | Tipo=AT | Campos PPO=8 | Trazabilidad: PPO=baseline; SAP/SF=datos de prueba hardcodeados en Main.xaml; reglas=recursos/gastos/compras prorrateados por anualidad, riesgos/garantia al ultimo mes, facturacion y realizado vacios; pendiente JP=revisar intercompany, externos y planificacion mensual. | AT: tarifas de venta reescaladas proporcionalmente para cuadrar venta facturable con importe total de venta del proyecto: 465.000,00 EUR. Se conservan horas, costes y perfiles; solo se ajusta tarifa de venta. Revisión requerida si negocio exige tarifa literal por linea PPO.</t>
+    <t>RPA_VALIDACION: Generado por RPA: 2026-05-12 02:50:02 | PPO=20251160543_PPO_CEducación_AMS_SI_Lote 2_v01.xlsm | NumeroSF=20251160543 | Tipo=AT | Campos PPO=8 | Trazabilidad: PPO=baseline; SAP/SF=datos de prueba hardcodeados en Main.xaml; reglas=recursos/gastos/compras prorrateados por anualidad, riesgos/garantia al ultimo mes, facturacion y realizado vacios; pendiente JP=revisar intercompany, externos y planificacion mensual. | AT: tarifas de venta reescaladas proporcionalmente para cuadrar venta facturable con importe total de venta del proyecto: 465.000,00 EUR. Se conservan horas, costes y perfiles; solo se ajusta tarifa de venta. Revisión requerida si negocio exige tarifa literal por linea PPO.</t>
   </si>
 </sst>
 </file>
@@ -3072,13 +3072,6 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -3088,9 +3081,16 @@
     <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="164" fontId="11" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -9016,7 +9016,7 @@
       </c>
       <c r="D4" s="315"/>
       <c r="E4" s="22"/>
-      <c r="F4" s="328" t="s">
+      <c r="F4" s="332" t="s">
         <v>238</v>
       </c>
       <c r="G4" s="333"/>
@@ -9029,26 +9029,26 @@
       <c r="J4" s="228" t="s">
         <v>241</v>
       </c>
-      <c r="K4" s="328" t="s">
+      <c r="K4" s="332" t="s">
         <v>242</v>
       </c>
-      <c r="L4" s="328"/>
-      <c r="M4" s="328"/>
-      <c r="N4" s="328"/>
+      <c r="L4" s="332"/>
+      <c r="M4" s="332"/>
+      <c r="N4" s="332"/>
     </row>
     <row r="5" spans="2:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="77" t="s">
         <v>243</v>
       </c>
-      <c r="C5" s="327" t="s">
+      <c r="C5" s="330" t="s">
         <v>244</v>
       </c>
-      <c r="D5" s="327"/>
+      <c r="D5" s="330"/>
       <c r="E5" s="22"/>
-      <c r="F5" s="327" t="s">
+      <c r="F5" s="330" t="s">
         <v>245</v>
       </c>
-      <c r="G5" s="327"/>
+      <c r="G5" s="330"/>
       <c r="H5" s="230">
         <v>0.5</v>
       </c>
@@ -9058,24 +9058,24 @@
       <c r="J5" s="289" t="s">
         <v>244</v>
       </c>
-      <c r="K5" s="327"/>
-      <c r="L5" s="327"/>
-      <c r="M5" s="327"/>
-      <c r="N5" s="327"/>
+      <c r="K5" s="330"/>
+      <c r="L5" s="330"/>
+      <c r="M5" s="330"/>
+      <c r="N5" s="330"/>
     </row>
     <row r="6" spans="2:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="77" t="s">
         <v>246</v>
       </c>
-      <c r="C6" s="327" t="s">
+      <c r="C6" s="330" t="s">
         <v>247</v>
       </c>
-      <c r="D6" s="327"/>
+      <c r="D6" s="330"/>
       <c r="E6" s="22"/>
-      <c r="F6" s="327" t="s">
+      <c r="F6" s="330" t="s">
         <v>248</v>
       </c>
-      <c r="G6" s="327"/>
+      <c r="G6" s="330"/>
       <c r="H6" s="230">
         <v>0.1</v>
       </c>
@@ -9083,26 +9083,26 @@
         <v>1000</v>
       </c>
       <c r="J6" s="289"/>
-      <c r="K6" s="327"/>
-      <c r="L6" s="327"/>
-      <c r="M6" s="327"/>
-      <c r="N6" s="327"/>
+      <c r="K6" s="330"/>
+      <c r="L6" s="330"/>
+      <c r="M6" s="330"/>
+      <c r="N6" s="330"/>
     </row>
     <row r="7" spans="2:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="77" t="s">
         <v>249</v>
       </c>
-      <c r="C7" s="332">
+      <c r="C7" s="331">
         <v>10000</v>
       </c>
-      <c r="D7" s="332"/>
+      <c r="D7" s="331"/>
       <c r="E7" s="229" t="s">
         <v>250</v>
       </c>
-      <c r="F7" s="327" t="s">
+      <c r="F7" s="330" t="s">
         <v>251</v>
       </c>
-      <c r="G7" s="327"/>
+      <c r="G7" s="330"/>
       <c r="H7" s="230">
         <v>0.2</v>
       </c>
@@ -9110,18 +9110,18 @@
         <v>2000</v>
       </c>
       <c r="J7" s="289"/>
-      <c r="K7" s="327"/>
-      <c r="L7" s="327"/>
-      <c r="M7" s="327"/>
-      <c r="N7" s="327"/>
+      <c r="K7" s="330"/>
+      <c r="L7" s="330"/>
+      <c r="M7" s="330"/>
+      <c r="N7" s="330"/>
     </row>
     <row r="8" spans="2:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D8" s="22"/>
       <c r="E8" s="22"/>
-      <c r="F8" s="327" t="s">
+      <c r="F8" s="330" t="s">
         <v>252</v>
       </c>
-      <c r="G8" s="327"/>
+      <c r="G8" s="330"/>
       <c r="H8" s="230">
         <v>0.1</v>
       </c>
@@ -9129,18 +9129,18 @@
         <v>1000</v>
       </c>
       <c r="J8" s="289"/>
-      <c r="K8" s="327"/>
-      <c r="L8" s="327"/>
-      <c r="M8" s="327"/>
-      <c r="N8" s="327"/>
+      <c r="K8" s="330"/>
+      <c r="L8" s="330"/>
+      <c r="M8" s="330"/>
+      <c r="N8" s="330"/>
     </row>
     <row r="9" spans="2:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D9" s="22"/>
       <c r="E9" s="56"/>
-      <c r="F9" s="327" t="s">
+      <c r="F9" s="330" t="s">
         <v>253</v>
       </c>
-      <c r="G9" s="327"/>
+      <c r="G9" s="330"/>
       <c r="H9" s="230">
         <v>0.1</v>
       </c>
@@ -9148,10 +9148,10 @@
         <v>1000</v>
       </c>
       <c r="J9" s="289"/>
-      <c r="K9" s="327"/>
-      <c r="L9" s="327"/>
-      <c r="M9" s="327"/>
-      <c r="N9" s="327"/>
+      <c r="K9" s="330"/>
+      <c r="L9" s="330"/>
+      <c r="M9" s="330"/>
+      <c r="N9" s="330"/>
       <c r="O9" s="24"/>
       <c r="P9" s="24"/>
     </row>
@@ -10237,12 +10237,12 @@
       <c r="W45" s="21"/>
     </row>
     <row r="46" spans="2:23" s="89" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="329" t="s">
+      <c r="B46" s="327" t="s">
         <v>233</v>
       </c>
-      <c r="C46" s="329"/>
-      <c r="D46" s="329"/>
-      <c r="E46" s="329"/>
+      <c r="C46" s="327"/>
+      <c r="D46" s="327"/>
+      <c r="E46" s="327"/>
       <c r="F46" s="219">
         <f>SUM(F13:F45)</f>
         <v>3000</v>
@@ -10406,16 +10406,16 @@
       <c r="R55" s="24"/>
     </row>
     <row r="56" spans="2:22" ht="285.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="330" t="s">
+      <c r="B56" s="328" t="s">
         <v>85</v>
       </c>
-      <c r="C56" s="331"/>
-      <c r="D56" s="331"/>
-      <c r="E56" s="331"/>
-      <c r="F56" s="331"/>
-      <c r="G56" s="331"/>
-      <c r="H56" s="331"/>
-      <c r="I56" s="331"/>
+      <c r="C56" s="329"/>
+      <c r="D56" s="329"/>
+      <c r="E56" s="329"/>
+      <c r="F56" s="329"/>
+      <c r="G56" s="329"/>
+      <c r="H56" s="329"/>
+      <c r="I56" s="329"/>
       <c r="J56" s="173"/>
       <c r="K56" s="173"/>
       <c r="L56" s="173"/>
@@ -10429,6 +10429,16 @@
   </sheetData>
   <autoFilter ref="B12:E12" xr:uid="{F0215733-3491-41E7-AEDA-44D9E214180D}"/>
   <mergeCells count="19">
+    <mergeCell ref="K9:N9"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="K4:N4"/>
+    <mergeCell ref="K5:N5"/>
+    <mergeCell ref="K6:N6"/>
+    <mergeCell ref="K7:N7"/>
+    <mergeCell ref="K8:N8"/>
     <mergeCell ref="B46:E46"/>
     <mergeCell ref="B56:I56"/>
     <mergeCell ref="C4:D4"/>
@@ -10438,16 +10448,6 @@
     <mergeCell ref="F5:G5"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="C10:D10"/>
-    <mergeCell ref="K4:N4"/>
-    <mergeCell ref="K5:N5"/>
-    <mergeCell ref="K6:N6"/>
-    <mergeCell ref="K7:N7"/>
-    <mergeCell ref="K8:N8"/>
-    <mergeCell ref="K9:N9"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="C10">
@@ -43020,6 +43020,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005104B4C06FD53E4DA82687A05841D03F" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f48deddc6bffdc45fb3ed0ec71e33c6c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7dc5af80-ab8f-4cff-b7cb-3463b3238b39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a8808579f8fa9f9643be1385777e037d" ns2:_="">
     <xsd:import namespace="7dc5af80-ab8f-4cff-b7cb-3463b3238b39"/>
@@ -43193,22 +43208,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4453D5CC-2F3C-48AA-8382-954EB2322467}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{794A36B1-E557-480A-80A5-281FC452AC8A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F36A1B76-9E34-462B-9C68-1BC8027D2211}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -43226,23 +43243,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{794A36B1-E557-480A-80A5-281FC452AC8A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4453D5CC-2F3C-48AA-8382-954EB2322467}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{040b5de6-6e2e-46f2-bca1-507eb809bbf7}" enabled="1" method="Privileged" siteId="{56d7daaa-b378-45b3-aa11-af9402b401b9}" contentBits="0" removed="0"/>

</xml_diff>

<commit_message>
plan rendimiento - e5
</commit_message>
<xml_diff>
--- a/oportunidad-generar-core-main/data/output/CORE_AT_20251160543.xlsx
+++ b/oportunidad-generar-core-main/data/output/CORE_AT_20251160543.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aortega\.nuget\packages\oportunidad-generar-core-main\1.0.42-ep4\content\data\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aortega\.nuget\packages\oportunidad-generar-core-main\1.0.55-ep5\content\data\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEBFD36F-C143-4626-9695-30AC36614281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C655245-B8E8-4BD2-A880-F76F42DA43FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="669" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1126,7 +1126,7 @@
     <t/>
   </si>
   <si>
-    <t>RPA_VALIDACION: Generado por RPA: 2026-05-12 03:09:29 | PPO=20251160543_PPO_CEducación_AMS_SI_Lote 2_v01.xlsm | NumeroSF=20251160543 | Tipo=AT | Campos PPO=8 | Trazabilidad: PPO=baseline; SAP/SF=datos de prueba hardcodeados en Main.xaml; reglas=recursos/gastos/compras prorrateados por anualidad, riesgos/garantia al ultimo mes, facturacion y realizado vacios; pendiente JP=revisar intercompany, externos y planificacion mensual. | AT: tarifas de venta reescaladas proporcionalmente para cuadrar venta facturable con importe total de venta del proyecto: 465.000,00 EUR. Se conservan horas, costes y perfiles; solo se ajusta tarifa de venta. Revisión requerida si negocio exige tarifa literal por linea PPO.</t>
+    <t>RPA_VALIDACION: Generado por RPA: 2026-05-12 04:28:50 | PPO=20251160543_PPO_CEducación_AMS_SI_Lote 2_v01.xlsm | NumeroSF=20251160543 | Tipo=AT | Campos PPO=8 | Trazabilidad: PPO=baseline; SAP/SF=datos de prueba hardcodeados en Main.xaml; reglas=recursos/gastos/compras prorrateados por anualidad, riesgos/garantia al ultimo mes, facturacion y realizado vacios; pendiente JP=revisar intercompany, externos y planificacion mensual. | AT: tarifas de venta reescaladas proporcionalmente para cuadrar venta facturable con importe total de venta del proyecto: 465.000,00 EUR. Se conservan horas, costes y perfiles; solo se ajusta tarifa de venta. Revisión requerida si negocio exige tarifa literal por linea PPO.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
plan rendimiento - e6
</commit_message>
<xml_diff>
--- a/oportunidad-generar-core-main/data/output/CORE_AT_20251160543.xlsx
+++ b/oportunidad-generar-core-main/data/output/CORE_AT_20251160543.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aortega\.nuget\packages\oportunidad-generar-core-main\1.0.55-ep5\content\data\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aortega\.nuget\packages\oportunidad-generar-core-main\1.0.56-ep6\content\data\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C655245-B8E8-4BD2-A880-F76F42DA43FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98A4FD6B-354F-45C0-9854-A6C05D165D4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="669" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1126,7 +1126,7 @@
     <t/>
   </si>
   <si>
-    <t>RPA_VALIDACION: Generado por RPA: 2026-05-12 04:28:50 | PPO=20251160543_PPO_CEducación_AMS_SI_Lote 2_v01.xlsm | NumeroSF=20251160543 | Tipo=AT | Campos PPO=8 | Trazabilidad: PPO=baseline; SAP/SF=datos de prueba hardcodeados en Main.xaml; reglas=recursos/gastos/compras prorrateados por anualidad, riesgos/garantia al ultimo mes, facturacion y realizado vacios; pendiente JP=revisar intercompany, externos y planificacion mensual. | AT: tarifas de venta reescaladas proporcionalmente para cuadrar venta facturable con importe total de venta del proyecto: 465.000,00 EUR. Se conservan horas, costes y perfiles; solo se ajusta tarifa de venta. Revisión requerida si negocio exige tarifa literal por linea PPO.</t>
+    <t>RPA_VALIDACION: Generado por RPA: 2026-05-12 04:40:41 | PPO=20251160543_PPO_CEducación_AMS_SI_Lote 2_v01.xlsm | NumeroSF=20251160543 | Tipo=AT | Campos PPO=8 | Trazabilidad: PPO=baseline; SAP/SF=datos de prueba hardcodeados en Main.xaml; reglas=recursos/gastos/compras prorrateados por anualidad, riesgos/garantia al ultimo mes, facturacion y realizado vacios; pendiente JP=revisar intercompany, externos y planificacion mensual. | AT: tarifas de venta reescaladas proporcionalmente para cuadrar venta facturable con importe total de venta del proyecto: 465.000,00 EUR. Se conservan horas, costes y perfiles; solo se ajusta tarifa de venta. Revisión requerida si negocio exige tarifa literal por linea PPO.</t>
   </si>
 </sst>
 </file>

</xml_diff>